<commit_message>
Update inventory for karwan - 1782482908813
</commit_message>
<xml_diff>
--- a/stores/karwan.xlsx
+++ b/stores/karwan.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Sno</t>
   </si>
@@ -30,6 +30,21 @@
   </si>
   <si>
     <t>Location</t>
+  </si>
+  <si>
+    <t>6924526310020</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -92,7 +107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
@@ -123,6 +138,26 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Update inventory for karwan - 1782484617664
</commit_message>
<xml_diff>
--- a/stores/karwan.xlsx
+++ b/stores/karwan.xlsx
@@ -32,19 +32,19 @@
     <t>Location</t>
   </si>
   <si>
-    <t>6924526310020</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>12</t>
+    <t>8886467080074</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t/>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>1-2-3</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update inventory for karwan - 1782485724245
</commit_message>
<xml_diff>
--- a/stores/karwan.xlsx
+++ b/stores/karwan.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Sno</t>
   </si>
@@ -30,21 +30,6 @@
   </si>
   <si>
     <t>Location</t>
-  </si>
-  <si>
-    <t>8886467080074</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>1-2-3</t>
   </si>
 </sst>
 </file>
@@ -96,9 +81,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyNumberFormat="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -107,11 +93,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
-    <col min="2" max="2" width="23.4375" customWidth="true"/>
+    <col min="2" max="2" width="31.25" customWidth="true"/>
     <col min="3" max="3" width="15.625" customWidth="true"/>
     <col min="4" max="4" width="15.625" customWidth="true"/>
     <col min="5" max="5" width="15.625" customWidth="true"/>
@@ -119,43 +105,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="1">
+      <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="1">
+      <c r="B1" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="1">
+      <c r="C1" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="1">
+      <c r="D1" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="1">
+      <c r="E1" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="1">
+      <c r="F1" t="s" s="2">
         <v>5</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update inventory for karwan - 1782485830909
</commit_message>
<xml_diff>
--- a/stores/karwan.xlsx
+++ b/stores/karwan.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Sno</t>
   </si>
@@ -30,6 +30,33 @@
   </si>
   <si>
     <t>Location</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>8886467080074</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2-3-1</t>
+  </si>
+  <si>
+    <t>6924526310020</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>3-6-4</t>
   </si>
 </sst>
 </file>
@@ -93,7 +120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
@@ -124,6 +151,46 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Update inventory for karwan - 1782493546083
</commit_message>
<xml_diff>
--- a/stores/karwan.xlsx
+++ b/stores/karwan.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>Sno</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>3-6-4</t>
+  </si>
+  <si>
+    <t>50219056</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>5-4-3</t>
   </si>
 </sst>
 </file>
@@ -111,7 +120,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyNumberFormat="true">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyNumberFormat="true">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -120,7 +129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.71875" customWidth="true"/>
@@ -191,6 +200,26 @@
         <v>14</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>